<commit_message>
Sync Plan_Campanas workbook costs with the published site
Two campaign cost cells in Plan_Campanas_Doner_Street_2027_Ajustado.xlsx
were stale leftovers from before an earlier correction pass: Google
Business Profile showed $1,200,000 instead of the published $500,000, and
Corporate Lunches showed $4,000,000 instead of $2,900,000. Their ROI 2027
values were already correct (computed from the right figures), only the
Costo total 2027 cells hadn't been updated to match. Fixed both so the
workbook's total ($47,600,000) matches the site's Marketing Campaign Plan
and Cost/Benefit sections exactly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Plan_Campanas_Doner_Street_2027_Ajustado.xlsx
+++ b/Plan_Campanas_Doner_Street_2027_Ajustado.xlsx
@@ -851,7 +851,7 @@
       <c r="G7" s="24" t="n"/>
       <c r="H7" s="24" t="n"/>
       <c r="I7" s="38" t="n">
-        <v>1200000</v>
+        <v>500000</v>
       </c>
       <c r="J7" s="39" t="n">
         <v>5.4</v>
@@ -977,7 +977,7 @@
       <c r="G10" s="24" t="n"/>
       <c r="H10" s="24" t="n"/>
       <c r="I10" s="38" t="n">
-        <v>4000000</v>
+        <v>2900000</v>
       </c>
       <c r="J10" s="39" t="n">
         <v>3.389</v>

</xml_diff>